<commit_message>
Cleanup: Removed unnecessary Python files and duplicate data
</commit_message>
<xml_diff>
--- a/lighthouse_scores_summary.xlsx
+++ b/lighthouse_scores_summary.xlsx
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -637,7 +637,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -677,7 +677,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -909,7 +909,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -949,7 +949,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -981,7 +981,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
@@ -1101,7 +1101,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
@@ -1141,7 +1141,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -1181,7 +1181,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -1221,7 +1221,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
@@ -1301,7 +1301,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -1341,7 +1341,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26">
@@ -1453,7 +1453,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -1533,7 +1533,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31">
@@ -1653,7 +1653,7 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32">
@@ -1685,7 +1685,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
@@ -1765,7 +1765,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35">
@@ -1805,7 +1805,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39">
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="40">
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42">
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
@@ -2109,7 +2109,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44">
@@ -2149,7 +2149,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -2229,7 +2229,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="47">
@@ -2269,7 +2269,7 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -2389,7 +2389,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51">
@@ -2469,7 +2469,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
@@ -2549,7 +2549,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="55">
@@ -2589,7 +2589,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="56">
@@ -2629,7 +2629,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57">
@@ -2669,7 +2669,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="58">
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
@@ -2749,7 +2749,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
@@ -2789,7 +2789,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
     </row>
     <row r="61">
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="62">
@@ -2869,7 +2869,7 @@
         </is>
       </c>
       <c r="J62" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63">
@@ -2909,7 +2909,7 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64">
@@ -2949,7 +2949,7 @@
         </is>
       </c>
       <c r="J64" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65">
@@ -2989,7 +2989,7 @@
         </is>
       </c>
       <c r="J65" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66">
@@ -3029,7 +3029,7 @@
         </is>
       </c>
       <c r="J66" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="67">
@@ -3069,7 +3069,7 @@
         </is>
       </c>
       <c r="J67" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
@@ -3109,7 +3109,7 @@
         </is>
       </c>
       <c r="J68" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="69">
@@ -3149,7 +3149,7 @@
         </is>
       </c>
       <c r="J69" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="70">
@@ -3189,7 +3189,7 @@
         </is>
       </c>
       <c r="J70" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -3229,7 +3229,7 @@
         </is>
       </c>
       <c r="J71" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -3309,7 +3309,7 @@
         </is>
       </c>
       <c r="J73" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="74">
@@ -3349,7 +3349,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75">
@@ -3389,7 +3389,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="76">
@@ -3429,7 +3429,7 @@
         </is>
       </c>
       <c r="J76" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77">
@@ -3469,7 +3469,7 @@
         </is>
       </c>
       <c r="J77" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78">
@@ -3509,7 +3509,7 @@
         </is>
       </c>
       <c r="J78" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79">
@@ -3549,7 +3549,7 @@
         </is>
       </c>
       <c r="J79" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="J80" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
     </row>
     <row r="81">
@@ -3629,7 +3629,7 @@
         </is>
       </c>
       <c r="J81" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -3669,7 +3669,7 @@
         </is>
       </c>
       <c r="J82" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="83">
@@ -3709,7 +3709,7 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="84">
@@ -3749,7 +3749,7 @@
         </is>
       </c>
       <c r="J84" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="85">
@@ -3789,7 +3789,7 @@
         </is>
       </c>
       <c r="J85" t="n">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="86">
@@ -3829,7 +3829,7 @@
         </is>
       </c>
       <c r="J86" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="87">
@@ -3869,7 +3869,7 @@
         </is>
       </c>
       <c r="J87" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
     </row>
     <row r="88">
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="J88" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="J89" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="90">
@@ -3989,7 +3989,7 @@
         </is>
       </c>
       <c r="J90" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="91">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="J91" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="92">
@@ -4061,7 +4061,7 @@
         </is>
       </c>
       <c r="J92" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
     </row>
     <row r="93">
@@ -4101,7 +4101,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="94">
@@ -4141,7 +4141,7 @@
         </is>
       </c>
       <c r="J94" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="95">
@@ -4181,7 +4181,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -4221,7 +4221,7 @@
         </is>
       </c>
       <c r="J96" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="97">
@@ -4261,7 +4261,7 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
     </row>
     <row r="98">
@@ -4301,7 +4301,7 @@
         </is>
       </c>
       <c r="J98" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="99">
@@ -4341,7 +4341,7 @@
         </is>
       </c>
       <c r="J99" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="100">
@@ -4381,7 +4381,7 @@
         </is>
       </c>
       <c r="J100" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>